<commit_message>
F01: Reorg to main/supp layout, harmonize alpha and annotations
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_supplementary.xlsx
+++ b/04_Figures/F01/c_data/F01_supplementary.xlsx
@@ -10,20 +10,20 @@
     <sheet name="panel_A" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="panel_B" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="panel_C" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SUPP_panel_D" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SUPP_panel_E" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SUPP_panel_F" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="SUPP_panel_A" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SUPP_panel_B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SUPP_panel_C" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t xml:space="preserve">F01 — Figure 1 source data</t>
   </si>
   <si>
-    <t xml:space="preserve">Phenotype panels A–C (main) and SUPP panels D–F.</t>
+    <t xml:space="preserve">Phenotype panels A–C (main) and SUPP panels A–C.</t>
   </si>
   <si>
     <t xml:space="preserve">Sheet</t>
@@ -50,28 +50,22 @@
     <t xml:space="preserve">Panel C: VL ultrasound thickness paired t-test by age group</t>
   </si>
   <si>
-    <t xml:space="preserve">SUPP_panel_D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP Panel D: Deadlift 1RM pre/post comparison</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP_panel_E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP Panel E: Type II fiber cross-sectional area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP_panel_F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP Panel F: Type I fiber cross-sectional area</t>
-  </si>
-  <si>
-    <t xml:space="preserve">data_dictionary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Column definitions for each panel CSV</t>
+    <t xml:space="preserve">SUPP_panel_A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPP Panel A: Deadlift 1RM pre/post comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPP_panel_B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPP Panel B: Type II fiber cross-sectional area</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPP_panel_C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SUPP Panel C: Type I fiber cross-sectional area</t>
   </si>
   <si>
     <t xml:space="preserve">Group</t>
@@ -575,14 +569,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>17</v>
-      </c>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:B1"/>
@@ -609,30 +595,30 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="D1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>22</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B2" t="n">
         <v>17</v>
@@ -655,7 +641,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B3" t="n">
         <v>15</v>
@@ -700,39 +686,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="I1" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="n">
         <v>3.18997773779259</v>
@@ -758,10 +744,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
         <v>4.5719266262061</v>
@@ -787,10 +773,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
         <v>1.39246199094184</v>
@@ -836,39 +822,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="I1" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="n">
         <v>6.55900186025861</v>
@@ -894,10 +880,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
         <v>5.27132264595624</v>
@@ -923,10 +909,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
         <v>3.23928168359076</v>
@@ -972,39 +958,39 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="I1" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="n">
         <v>14.7688449703674</v>
@@ -1030,10 +1016,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
         <v>1.87694637635175</v>
@@ -1059,10 +1045,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
         <v>3.13448667481087</v>
@@ -1109,42 +1095,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="J1" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="n">
         <v>13</v>
@@ -1173,10 +1159,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>
@@ -1205,10 +1191,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
         <v>23</v>
@@ -1258,42 +1244,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="H1" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="J1" s="5" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C2" t="n">
         <v>13</v>
@@ -1322,10 +1308,10 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>
@@ -1354,10 +1340,10 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" t="n">
         <v>23</v>

</xml_diff>

<commit_message>
Pre-audit checkpoint: regenerated outputs + F06 restructure + style normalization
All figure outputs regenerated from current pipeline state. F06 main
restructured to 2-panel layout (panel_A heatmap + panel_B stacked
scatters). Brown module label updated (redox-glycolysis -> muscle
contraction). shared/style.R updated with J Physiol text hierarchy
(T1=7pt, T2=5pt, T3=4pt, Helvetica). F01-F07 panel scripts updated
to use FIG_THEME with journal-calibrated sizes. F02 intermediate
audit CSVs added (CV scatter, wilcoxon, imputed variability).
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_supplementary.xlsx
+++ b/04_Figures/F01/c_data/F01_supplementary.xlsx
@@ -10,9 +10,6 @@
     <sheet name="panel_A" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="panel_B" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="panel_C" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SUPP_panel_A" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SUPP_panel_B" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SUPP_panel_C" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -938,438 +935,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="n">
-        <v>14.7688449703674</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0.0000000000964241430155066</v>
-      </c>
-      <c r="E2" t="n">
-        <v>16</v>
-      </c>
-      <c r="F2" t="n">
-        <v>34.6428952706309</v>
-      </c>
-      <c r="G2" t="n">
-        <v>29.6702885832475</v>
-      </c>
-      <c r="H2" t="n">
-        <v>39.6155019580143</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.644086480755537</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1.87694637635175</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0.097361685383249</v>
-      </c>
-      <c r="E3" t="n">
-        <v>8</v>
-      </c>
-      <c r="F3" t="n">
-        <v>12.5042713332305</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-2.85839526473125</v>
-      </c>
-      <c r="H3" t="n">
-        <v>27.8669379311923</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.237257638742384</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="n">
-        <v>3.13448667481087</v>
-      </c>
-      <c r="D4" t="n">
-        <v>0.0105726137329648</v>
-      </c>
-      <c r="E4" t="n">
-        <v>10.0294265576391</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-22.1386239374004</v>
-      </c>
-      <c r="G4" t="n">
-        <v>6.40771726946544</v>
-      </c>
-      <c r="H4" t="n">
-        <v>37.8695306053354</v>
-      </c>
-      <c r="I4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="n">
-        <v>13</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.79441278568396</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.0162113506588155</v>
-      </c>
-      <c r="F2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" t="n">
-        <v>856.603728058635</v>
-      </c>
-      <c r="H2" t="n">
-        <v>188.706987034343</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1524.50046908293</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.629844097930084</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-1.12717233951929</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.288823381952292</v>
-      </c>
-      <c r="F3" t="n">
-        <v>9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-381.6</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-1147.44488729731</v>
-      </c>
-      <c r="I3" t="n">
-        <v>384.244887297309</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.166727557880152</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="n">
-        <v>23</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2.71115529634061</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.0135165137442106</v>
-      </c>
-      <c r="F4" t="n">
-        <v>19.8168408558481</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-1238.20372805863</v>
-      </c>
-      <c r="H4" t="n">
-        <v>284.96473107296</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2191.44272504431</v>
-      </c>
-      <c r="J4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="n">
-        <v>13</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.47802908436044</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.0290628558366825</v>
-      </c>
-      <c r="F2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" t="n">
-        <v>572.085261566636</v>
-      </c>
-      <c r="H2" t="n">
-        <v>69.0779661996328</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1075.09255693364</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.158997959578344</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-1.75727569644542</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.112745012158823</v>
-      </c>
-      <c r="F3" t="n">
-        <v>9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-722.6</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-1652.80962455947</v>
-      </c>
-      <c r="I3" t="n">
-        <v>207.609624559473</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.485336464164219</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="n">
-        <v>23</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2.74542435658255</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.015399032964439</v>
-      </c>
-      <c r="F4" t="n">
-        <v>14.4882690796857</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-1294.68526156664</v>
-      </c>
-      <c r="H4" t="n">
-        <v>286.436818157853</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2302.93370497542</v>
-      </c>
-      <c r="J4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix minor style issues + full pipeline verification run
Code fixes (4 files):
- shared/style.R: resolve tag size conflict (plot.tag now uses BASE_TAG=8)
- F06/panel_B.R: update header from PILOT to production
- F01/supp/panel_A.R: fmt_p -> fmt_p_plot with parse=TRUE (3 locations)
- F04/rrho_manual.R: archive dead code (294 lines, never sourced)

Infrastructure:
- .Rprofile: remove broken renv reference
- A_YvO_2025.Rproj: create for rprojroot (was gitignored, needed for CLI runs)

Full pipeline run verified (all stages, zero errors):
  01_normalization: 2113 proteins x 62 samples
  02_Imputation: missForest OOB=0.1088
  03_DEP: 196 Aging Pi, 100 TY, 18 TO, 34 Int (all match expected)
  F00-F07: all composites + xlsx regenerated successfully
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_supplementary.xlsx
+++ b/04_Figures/F01/c_data/F01_supplementary.xlsx
@@ -10,6 +10,9 @@
     <sheet name="panel_A" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="panel_B" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="panel_C" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SUPP_panel_A" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SUPP_panel_B" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SUPP_panel_C" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -935,4 +938,438 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="n">
+        <v>14.7688449703674</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.0000000000964241430155066</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F2" t="n">
+        <v>34.6428952706309</v>
+      </c>
+      <c r="G2" t="n">
+        <v>29.6702885832475</v>
+      </c>
+      <c r="H2" t="n">
+        <v>39.6155019580143</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.644086480755537</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1.87694637635175</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.097361685383249</v>
+      </c>
+      <c r="E3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F3" t="n">
+        <v>12.5042713332305</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-2.85839526473125</v>
+      </c>
+      <c r="H3" t="n">
+        <v>27.8669379311923</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.237257638742384</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3.13448667481087</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.0105726137329648</v>
+      </c>
+      <c r="E4" t="n">
+        <v>10.0294265576391</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-22.1386239374004</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6.40771726946544</v>
+      </c>
+      <c r="H4" t="n">
+        <v>37.8695306053354</v>
+      </c>
+      <c r="I4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.79441278568396</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0162113506588155</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" t="n">
+        <v>856.603728058635</v>
+      </c>
+      <c r="H2" t="n">
+        <v>188.706987034343</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1524.50046908293</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.629844097930084</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1.12717233951929</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.288823381952292</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-381.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-1147.44488729731</v>
+      </c>
+      <c r="I3" t="n">
+        <v>384.244887297309</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.166727557880152</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.71115529634061</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0135165137442106</v>
+      </c>
+      <c r="F4" t="n">
+        <v>19.8168408558481</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-1238.20372805863</v>
+      </c>
+      <c r="H4" t="n">
+        <v>284.96473107296</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2191.44272504431</v>
+      </c>
+      <c r="J4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <cols>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="n">
+        <v>13</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2.47802908436044</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.0290628558366825</v>
+      </c>
+      <c r="F2" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" t="n">
+        <v>572.085261566636</v>
+      </c>
+      <c r="H2" t="n">
+        <v>69.0779661996328</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1075.09255693364</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.158997959578344</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1.75727569644542</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.112745012158823</v>
+      </c>
+      <c r="F3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-722.6</v>
+      </c>
+      <c r="H3" t="n">
+        <v>-1652.80962455947</v>
+      </c>
+      <c r="I3" t="n">
+        <v>207.609624559473</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.485336464164219</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D4" t="n">
+        <v>2.74542435658255</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.015399032964439</v>
+      </c>
+      <c r="F4" t="n">
+        <v>14.4882690796857</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-1294.68526156664</v>
+      </c>
+      <c r="H4" t="n">
+        <v>286.436818157853</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2302.93370497542</v>
+      </c>
+      <c r="J4"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
F01: phenotype figure panel and layout updates
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_supplementary.xlsx
+++ b/04_Figures/F01/c_data/F01_supplementary.xlsx
@@ -675,13 +675,14 @@
   <cols>
     <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -692,24 +693,27 @@
         <v>16</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -721,24 +725,27 @@
         <v>23</v>
       </c>
       <c r="C2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D2" t="n">
         <v>3.18997773779259</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.00569641165229446</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>16</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>2.20941176470588</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.741143302304994</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>3.67768022710677</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.0589546260567265</v>
       </c>
     </row>
@@ -750,24 +757,27 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
         <v>4.5719266262061</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.0004351155884287</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>14</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>1.18017345392857</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.62652932960883</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>1.7338175782483</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.308889212998157</v>
       </c>
     </row>
@@ -779,24 +789,27 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D4" t="n">
         <v>1.39246199094184</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.178844473519128</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>20.3058830697667</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-1.02923831077732</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>-0.511114019968263</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>2.5695906415229</v>
       </c>
-      <c r="I4"/>
+      <c r="J4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -811,13 +824,14 @@
   <cols>
     <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -828,24 +842,27 @@
         <v>16</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -857,24 +874,27 @@
         <v>23</v>
       </c>
       <c r="C2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D2" t="n">
         <v>6.55900186025861</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.00000657814233487256</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>16</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>0.46764705882353</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>0.316500969938879</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>0.61879314770818</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.154019706948298</v>
       </c>
     </row>
@@ -886,24 +906,27 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
         <v>5.27132264595624</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.00011816977551927</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>14</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>0.204666666666667</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>0.121392245499539</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>0.287941087833794</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.628876363010418</v>
       </c>
     </row>
@@ -915,24 +938,27 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D4" t="n">
         <v>3.23928168359076</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.00343861635736173</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>24.4402387953263</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-0.262980392156863</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>0.0955828026178479</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>0.430377981695878</v>
       </c>
-      <c r="I4"/>
+      <c r="J4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -947,13 +973,14 @@
   <cols>
     <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -964,24 +991,27 @@
         <v>16</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="E1" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="J1" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -993,24 +1023,27 @@
         <v>23</v>
       </c>
       <c r="C2" t="n">
+        <v>17</v>
+      </c>
+      <c r="D2" t="n">
         <v>14.7688449703674</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>0.0000000000964241430155066</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
         <v>16</v>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>34.6428952706309</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>29.6702885832475</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>39.6155019580143</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>0.644086480755537</v>
       </c>
     </row>
@@ -1022,24 +1055,27 @@
         <v>24</v>
       </c>
       <c r="C3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D3" t="n">
         <v>1.87694637635175</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>0.097361685383249</v>
       </c>
-      <c r="E3" t="n">
+      <c r="F3" t="n">
         <v>8</v>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>12.5042713332305</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>-2.85839526473125</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>27.8669379311923</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>0.237257638742384</v>
       </c>
     </row>
@@ -1051,24 +1087,27 @@
         <v>35</v>
       </c>
       <c r="C4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D4" t="n">
         <v>3.13448667481087</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>0.0105726137329648</v>
       </c>
-      <c r="E4" t="n">
+      <c r="F4" t="n">
         <v>10.0294265576391</v>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>-22.1386239374004</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>6.40771726946544</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>37.8695306053354</v>
       </c>
-      <c r="I4"/>
+      <c r="J4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Tighten pipeline scripts and update README
- Remove dead code: unused subtitle assignments (F03), no-op ifelse and
  dead export variables (F04/F05 ORA panels), unused time_binary (F06
  hub), duplicate enrichment CSV write (F06 WGCNA run), duplicate xlsx
  sheet reference (F06 stitcher)
- Delete stale file: wgcna_module_GO_enrichment.csv (was identical to
  wgcna_module_enrichment.csv)
- Route S01-S03 Box copies from 03_Supplementary/ root into tables/
  subdirectory with S0X_Table_* naming to match S04-S11 convention
- Re-run stages 01-03 report scripts to deliver fresh copies
- Add manuscript outputs section to README with paths for all 7 main
  figures, 9 supplementary figures, and 11 supplementary tables
- Regenerated pipeline outputs (PDF timestamps differ; PNGs and data
  artifacts verified against pre-run snapshots)
</commit_message>
<xml_diff>
--- a/04_Figures/F01/c_data/F01_supplementary.xlsx
+++ b/04_Figures/F01/c_data/F01_supplementary.xlsx
@@ -6,67 +6,18 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="panel_A" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="panel_B" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="panel_C" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="SUPP_panel_A" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="SUPP_panel_B" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="SUPP_panel_C" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="panel_A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="panel_B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="panel_C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="SUPP_panel_A" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SUPP_panel_B" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="SUPP_panel_C" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
-  <si>
-    <t xml:space="preserve">F01 — Phenotype source data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Main panels A–C and supplementary panels A–C.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sheet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description</t>
-  </si>
-  <si>
-    <t xml:space="preserve">panel_A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training volume</t>
-  </si>
-  <si>
-    <t xml:space="preserve">panel_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DXA LBM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">panel_C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VL thickness</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP_panel_A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Deadlift 1RM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP_panel_B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type II fCSA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SUPP_panel_C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type I fCSA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t xml:space="preserve">Group</t>
   </si>
@@ -133,7 +84,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -142,46 +93,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF555555"/>
-      <name val="Calibri"/>
-      <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <b/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <b/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2F4F4F"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -196,19 +119,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -499,81 +412,85 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="32.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="95.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="3.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" ht="40" customHeight="1">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="4" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="s">
+      <c r="B2" t="n">
+        <v>15</v>
+      </c>
+      <c r="C2" t="n">
+        <v>211904.046228677</v>
+      </c>
+      <c r="D2" t="n">
+        <v>63961.6607283764</v>
+      </c>
+      <c r="E2" t="n">
+        <v>16514.8297864514</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.988399773207149</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.770720835814133</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>15</v>
+      <c r="B3" t="n">
+        <v>17</v>
+      </c>
+      <c r="C3" t="n">
+        <v>217658.101764706</v>
+      </c>
+      <c r="D3" t="n">
+        <v>42922.5057447456</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10410.2367589275</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.505766491328304</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.770720835814133</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="A2:B2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
@@ -584,83 +501,143 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
-    <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="3.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="11.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>22</v>
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" t="n">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>211904.046228677</v>
+        <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>63961.6607283764</v>
+        <v>3.18997773779259</v>
       </c>
       <c r="E2" t="n">
-        <v>16514.8297864514</v>
+        <v>0.00569641165229446</v>
       </c>
       <c r="F2" t="n">
-        <v>0.988399773207149</v>
+        <v>16</v>
       </c>
       <c r="G2" t="n">
-        <v>0.770720835814133</v>
+        <v>2.20941176470588</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.741143302304994</v>
+      </c>
+      <c r="I2" t="n">
+        <v>3.67768022710677</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.0589546260567265</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" t="n">
         <v>17</v>
       </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
       <c r="C3" t="n">
-        <v>217658.101764706</v>
+        <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>42922.5057447456</v>
+        <v>4.5719266262061</v>
       </c>
       <c r="E3" t="n">
-        <v>10410.2367589275</v>
+        <v>0.0004351155884287</v>
       </c>
       <c r="F3" t="n">
-        <v>0.505766491328304</v>
+        <v>14</v>
       </c>
       <c r="G3" t="n">
-        <v>0.770720835814133</v>
-      </c>
+        <v>1.18017345392857</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.62652932960883</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1.7338175782483</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.308889212998157</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1.39246199094184</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.178844473519128</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20.3058830697667</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-1.02923831077732</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-0.511114019968263</v>
+      </c>
+      <c r="I4" t="n">
+        <v>2.5695906415229</v>
+      </c>
+      <c r="J4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -686,128 +663,128 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
         <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>3.18997773779259</v>
+        <v>6.55900186025861</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00569641165229446</v>
+        <v>0.00000657814233487256</v>
       </c>
       <c r="F2" t="n">
         <v>16</v>
       </c>
       <c r="G2" t="n">
-        <v>2.20941176470588</v>
+        <v>0.46764705882353</v>
       </c>
       <c r="H2" t="n">
-        <v>0.741143302304994</v>
+        <v>0.316500969938879</v>
       </c>
       <c r="I2" t="n">
-        <v>3.67768022710677</v>
+        <v>0.61879314770818</v>
       </c>
       <c r="J2" t="n">
-        <v>0.0589546260567265</v>
+        <v>0.154019706948298</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
         <v>15</v>
       </c>
       <c r="D3" t="n">
-        <v>4.5719266262061</v>
+        <v>5.27132264595624</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0004351155884287</v>
+        <v>0.00011816977551927</v>
       </c>
       <c r="F3" t="n">
         <v>14</v>
       </c>
       <c r="G3" t="n">
-        <v>1.18017345392857</v>
+        <v>0.204666666666667</v>
       </c>
       <c r="H3" t="n">
-        <v>0.62652932960883</v>
+        <v>0.121392245499539</v>
       </c>
       <c r="I3" t="n">
-        <v>1.7338175782483</v>
+        <v>0.287941087833794</v>
       </c>
       <c r="J3" t="n">
-        <v>0.308889212998157</v>
+        <v>0.628876363010418</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
         <v>32</v>
       </c>
       <c r="D4" t="n">
-        <v>1.39246199094184</v>
+        <v>3.23928168359076</v>
       </c>
       <c r="E4" t="n">
-        <v>0.178844473519128</v>
+        <v>0.00343861635736173</v>
       </c>
       <c r="F4" t="n">
-        <v>20.3058830697667</v>
+        <v>24.4402387953263</v>
       </c>
       <c r="G4" t="n">
-        <v>-1.02923831077732</v>
+        <v>-0.262980392156863</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.511114019968263</v>
+        <v>0.0955828026178479</v>
       </c>
       <c r="I4" t="n">
-        <v>2.5695906415229</v>
+        <v>0.430377981695878</v>
       </c>
       <c r="J4"/>
     </row>
@@ -835,128 +812,128 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
         <v>17</v>
       </c>
       <c r="D2" t="n">
-        <v>6.55900186025861</v>
+        <v>14.7688449703674</v>
       </c>
       <c r="E2" t="n">
-        <v>0.00000657814233487256</v>
+        <v>0.0000000000964241430155066</v>
       </c>
       <c r="F2" t="n">
         <v>16</v>
       </c>
       <c r="G2" t="n">
-        <v>0.46764705882353</v>
+        <v>34.6428952706309</v>
       </c>
       <c r="H2" t="n">
-        <v>0.316500969938879</v>
+        <v>29.6702885832475</v>
       </c>
       <c r="I2" t="n">
-        <v>0.61879314770818</v>
+        <v>39.6155019580143</v>
       </c>
       <c r="J2" t="n">
-        <v>0.154019706948298</v>
+        <v>0.644086480755537</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D3" t="n">
-        <v>5.27132264595624</v>
+        <v>1.87694637635175</v>
       </c>
       <c r="E3" t="n">
-        <v>0.00011816977551927</v>
+        <v>0.097361685383249</v>
       </c>
       <c r="F3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
-        <v>0.204666666666667</v>
+        <v>12.5042713332305</v>
       </c>
       <c r="H3" t="n">
-        <v>0.121392245499539</v>
+        <v>-2.85839526473125</v>
       </c>
       <c r="I3" t="n">
-        <v>0.287941087833794</v>
+        <v>27.8669379311923</v>
       </c>
       <c r="J3" t="n">
-        <v>0.628876363010418</v>
+        <v>0.237257638742384</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D4" t="n">
-        <v>3.23928168359076</v>
+        <v>3.13448667481087</v>
       </c>
       <c r="E4" t="n">
-        <v>0.00343861635736173</v>
+        <v>0.0105726137329648</v>
       </c>
       <c r="F4" t="n">
-        <v>24.4402387953263</v>
+        <v>10.0294265576391</v>
       </c>
       <c r="G4" t="n">
-        <v>-0.262980392156863</v>
+        <v>-22.1386239374004</v>
       </c>
       <c r="H4" t="n">
-        <v>0.0955828026178479</v>
+        <v>6.40771726946544</v>
       </c>
       <c r="I4" t="n">
-        <v>0.430377981695878</v>
+        <v>37.8695306053354</v>
       </c>
       <c r="J4"/>
     </row>
@@ -984,128 +961,128 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>14.7688449703674</v>
+        <v>2.79441278568396</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0000000000964241430155066</v>
+        <v>0.0162113506588155</v>
       </c>
       <c r="F2" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G2" t="n">
-        <v>34.6428952706309</v>
+        <v>856.603728058635</v>
       </c>
       <c r="H2" t="n">
-        <v>29.6702885832475</v>
+        <v>188.706987034343</v>
       </c>
       <c r="I2" t="n">
-        <v>39.6155019580143</v>
+        <v>1524.50046908293</v>
       </c>
       <c r="J2" t="n">
-        <v>0.644086480755537</v>
+        <v>0.629844097930084</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-1.12717233951929</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.288823381952292</v>
+      </c>
+      <c r="F3" t="n">
         <v>9</v>
       </c>
-      <c r="D3" t="n">
-        <v>1.87694637635175</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.097361685383249</v>
-      </c>
-      <c r="F3" t="n">
-        <v>8</v>
-      </c>
       <c r="G3" t="n">
-        <v>12.5042713332305</v>
+        <v>-381.6</v>
       </c>
       <c r="H3" t="n">
-        <v>-2.85839526473125</v>
+        <v>-1147.44488729731</v>
       </c>
       <c r="I3" t="n">
-        <v>27.8669379311923</v>
+        <v>384.244887297309</v>
       </c>
       <c r="J3" t="n">
-        <v>0.237257638742384</v>
+        <v>0.166727557880152</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
-        <v>3.13448667481087</v>
+        <v>2.71115529634061</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0105726137329648</v>
+        <v>0.0135165137442106</v>
       </c>
       <c r="F4" t="n">
-        <v>10.0294265576391</v>
+        <v>19.8168408558481</v>
       </c>
       <c r="G4" t="n">
-        <v>-22.1386239374004</v>
+        <v>-1238.20372805863</v>
       </c>
       <c r="H4" t="n">
-        <v>6.40771726946544</v>
+        <v>284.96473107296</v>
       </c>
       <c r="I4" t="n">
-        <v>37.8695306053354</v>
+        <v>2191.44272504431</v>
       </c>
       <c r="J4"/>
     </row>
@@ -1133,256 +1110,107 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
+      <c r="A1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="C2" t="n">
         <v>13</v>
       </c>
       <c r="D2" t="n">
-        <v>2.79441278568396</v>
+        <v>2.47802908436044</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0162113506588155</v>
+        <v>0.0290628558366825</v>
       </c>
       <c r="F2" t="n">
         <v>12</v>
       </c>
       <c r="G2" t="n">
-        <v>856.603728058635</v>
+        <v>572.085261566636</v>
       </c>
       <c r="H2" t="n">
-        <v>188.706987034343</v>
+        <v>69.0779661996328</v>
       </c>
       <c r="I2" t="n">
-        <v>1524.50046908293</v>
+        <v>1075.09255693364</v>
       </c>
       <c r="J2" t="n">
-        <v>0.629844097930084</v>
+        <v>0.158997959578344</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="C3" t="n">
         <v>10</v>
       </c>
       <c r="D3" t="n">
-        <v>-1.12717233951929</v>
+        <v>-1.75727569644542</v>
       </c>
       <c r="E3" t="n">
-        <v>0.288823381952292</v>
+        <v>0.112745012158823</v>
       </c>
       <c r="F3" t="n">
         <v>9</v>
       </c>
       <c r="G3" t="n">
-        <v>-381.6</v>
+        <v>-722.6</v>
       </c>
       <c r="H3" t="n">
-        <v>-1147.44488729731</v>
+        <v>-1652.80962455947</v>
       </c>
       <c r="I3" t="n">
-        <v>384.244887297309</v>
+        <v>207.609624559473</v>
       </c>
       <c r="J3" t="n">
-        <v>0.166727557880152</v>
+        <v>0.485336464164219</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" t="n">
-        <v>23</v>
-      </c>
-      <c r="D4" t="n">
-        <v>2.71115529634061</v>
-      </c>
-      <c r="E4" t="n">
-        <v>0.0135165137442106</v>
-      </c>
-      <c r="F4" t="n">
-        <v>19.8168408558481</v>
-      </c>
-      <c r="G4" t="n">
-        <v>-1238.20372805863</v>
-      </c>
-      <c r="H4" t="n">
-        <v>284.96473107296</v>
-      </c>
-      <c r="I4" t="n">
-        <v>2191.44272504431</v>
-      </c>
-      <c r="J4"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
-  <cols>
-    <col min="1" max="1" width="16.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="12.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="3.71" hidden="0" customWidth="1"/>
-    <col min="4" max="4" width="11.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="11.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="11.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="11.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="11.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="11.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="11.71" hidden="0" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" t="n">
-        <v>13</v>
-      </c>
-      <c r="D2" t="n">
-        <v>2.47802908436044</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0.0290628558366825</v>
-      </c>
-      <c r="F2" t="n">
-        <v>12</v>
-      </c>
-      <c r="G2" t="n">
-        <v>572.085261566636</v>
-      </c>
-      <c r="H2" t="n">
-        <v>69.0779661996328</v>
-      </c>
-      <c r="I2" t="n">
-        <v>1075.09255693364</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.158997959578344</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C3" t="n">
-        <v>10</v>
-      </c>
-      <c r="D3" t="n">
-        <v>-1.75727569644542</v>
-      </c>
-      <c r="E3" t="n">
-        <v>0.112745012158823</v>
-      </c>
-      <c r="F3" t="n">
-        <v>9</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-722.6</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-1652.80962455947</v>
-      </c>
-      <c r="I3" t="n">
-        <v>207.609624559473</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.485336464164219</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="C4" t="n">
         <v>23</v>

</xml_diff>